<commit_message>
Added Excel utilities and day41-day44 practice
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://orange0-my.sharepoint.com/personal/himanshu1_mishra_orange_com/Documents/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="11_F25DC773A252ABDACC1048C78198483A5BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61619E37-7AB0-4726-8640-349A04541E46}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5BF28178-3BAB-4D1E-84DB-C85F9FE3A278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -406,8 +402,8 @@
   <cols>
     <col min="1" max="1" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>